<commit_message>
Update attendees for quiz: my-quiz — fejinfm2000@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/my-quiz/attendees.xlsx
+++ b/quizzes/my-quiz/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -455,9 +455,50 @@
         <v>Grade</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fejinfm2000@gmail.com</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Fejin FM</v>
+      </c>
+      <c r="C2" t="str">
+        <v>my quiz</v>
+      </c>
+      <c r="D2" t="str">
+        <v>3/18/2026, 12:20:47 AM</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="L2" t="str">
+        <v>100.00</v>
+      </c>
+      <c r="M2" t="str">
+        <v>A+</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: my-quiz — fejinfm000@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/my-quiz/attendees.xlsx
+++ b/quizzes/my-quiz/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -496,9 +496,50 @@
         <v>A+</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fejinfm000@gmail.com</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Fejin FM</v>
+      </c>
+      <c r="C3" t="str">
+        <v>my quiz</v>
+      </c>
+      <c r="D3" t="str">
+        <v>3/18/2026, 12:21:38 AM</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="M3" t="str">
+        <v>F</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: my-quiz — chinnaduraip@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/my-quiz/attendees.xlsx
+++ b/quizzes/my-quiz/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -466,7 +466,7 @@
         <v>my quiz</v>
       </c>
       <c r="D2" t="str">
-        <v>18/03/2026, 00:21:38</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -507,7 +507,7 @@
         <v>my quiz</v>
       </c>
       <c r="D3" t="str">
-        <v>18/03/2026, 07:45:02</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -534,12 +534,53 @@
         <v>50.00</v>
       </c>
       <c r="M3" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>chinnaduraip@gmail.com</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Chinna</v>
+      </c>
+      <c r="C4" t="str">
+        <v>my quiz</v>
+      </c>
+      <c r="D4" t="str">
+        <v>18/3/2026, 10:12:40 am</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" t="str">
+        <v>50.00</v>
+      </c>
+      <c r="M4" t="str">
         <v>D</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: my-quiz — admin@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/my-quiz/attendees.xlsx
+++ b/quizzes/my-quiz/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -548,7 +548,7 @@
         <v>my quiz</v>
       </c>
       <c r="D4" t="str">
-        <v>18/3/2026, 10:12:40 am</v>
+        <v>Invalid Date</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -575,12 +575,53 @@
         <v>50.00</v>
       </c>
       <c r="M4" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>admin@gmail.com</v>
+      </c>
+      <c r="B5" t="str">
+        <v>admin</v>
+      </c>
+      <c r="C5" t="str">
+        <v>my quiz</v>
+      </c>
+      <c r="D5" t="str">
+        <v>18/3/2026, 2:37:47 pm</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5" t="str">
+        <v>50.00</v>
+      </c>
+      <c r="M5" t="str">
         <v>D</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: my-quiz — jess@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/my-quiz/attendees.xlsx
+++ b/quizzes/my-quiz/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -619,9 +619,50 @@
         <v>D</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>jess@gmail.com</v>
+      </c>
+      <c r="B6" t="str">
+        <v>jess</v>
+      </c>
+      <c r="C6" t="str">
+        <v>my quiz</v>
+      </c>
+      <c r="D6" t="str">
+        <v>3/23/2026, 8:04:19 PM</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6" t="str">
+        <v>50.00</v>
+      </c>
+      <c r="M6" t="str">
+        <v>D</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update attendees for quiz: my-quiz — charanm@clarium.tech
</commit_message>
<xml_diff>
--- a/quizzes/my-quiz/attendees.xlsx
+++ b/quizzes/my-quiz/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -660,9 +660,50 @@
         <v>D</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>charanm@clarium.tech</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Charan M</v>
+      </c>
+      <c r="C7" t="str">
+        <v>my quiz</v>
+      </c>
+      <c r="D7" t="str">
+        <v>3/27/2026, 4:13:11 PM</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="str">
+        <v>50.00</v>
+      </c>
+      <c r="M7" t="str">
+        <v>D</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>